<commit_message>
Fix layover day-row off-by-one (Day1 = 18-Jul)
</commit_message>
<xml_diff>
--- a/uploads/HZ-ASD_C2_6Y_CABIN_WP_TRACKER.xlsx
+++ b/uploads/HZ-ASD_C2_6Y_CABIN_WP_TRACKER.xlsx
@@ -36955,807 +36955,807 @@
         </is>
       </c>
       <c r="D3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=1,"Day "&amp;1,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=0,"Day "&amp;1,"")</f>
         <v/>
       </c>
       <c r="F3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=2,"Day "&amp;2,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=1,"Day "&amp;2,"")</f>
         <v/>
       </c>
       <c r="H3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=3,"Day "&amp;3,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=2,"Day "&amp;3,"")</f>
         <v/>
       </c>
       <c r="J3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=4,"Day "&amp;4,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=3,"Day "&amp;4,"")</f>
         <v/>
       </c>
       <c r="L3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=5,"Day "&amp;5,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=4,"Day "&amp;5,"")</f>
         <v/>
       </c>
       <c r="N3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=6,"Day "&amp;6,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=5,"Day "&amp;6,"")</f>
         <v/>
       </c>
       <c r="P3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=7,"Day "&amp;7,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=6,"Day "&amp;7,"")</f>
         <v/>
       </c>
       <c r="R3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=8,"Day "&amp;8,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=7,"Day "&amp;8,"")</f>
         <v/>
       </c>
       <c r="T3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=9,"Day "&amp;9,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=8,"Day "&amp;9,"")</f>
         <v/>
       </c>
       <c r="V3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=10,"Day "&amp;10,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=9,"Day "&amp;10,"")</f>
         <v/>
       </c>
       <c r="X3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=11,"Day "&amp;11,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=10,"Day "&amp;11,"")</f>
         <v/>
       </c>
       <c r="Z3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=12,"Day "&amp;12,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=11,"Day "&amp;12,"")</f>
         <v/>
       </c>
       <c r="AB3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=13,"Day "&amp;13,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=12,"Day "&amp;13,"")</f>
         <v/>
       </c>
       <c r="AD3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=14,"Day "&amp;14,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=13,"Day "&amp;14,"")</f>
         <v/>
       </c>
       <c r="AF3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=15,"Day "&amp;15,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=14,"Day "&amp;15,"")</f>
         <v/>
       </c>
       <c r="AH3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=16,"Day "&amp;16,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=15,"Day "&amp;16,"")</f>
         <v/>
       </c>
       <c r="AJ3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=17,"Day "&amp;17,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=16,"Day "&amp;17,"")</f>
         <v/>
       </c>
       <c r="AL3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=18,"Day "&amp;18,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=17,"Day "&amp;18,"")</f>
         <v/>
       </c>
       <c r="AN3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=19,"Day "&amp;19,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=18,"Day "&amp;19,"")</f>
         <v/>
       </c>
       <c r="AP3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=20,"Day "&amp;20,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=19,"Day "&amp;20,"")</f>
         <v/>
       </c>
       <c r="AR3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=21,"Day "&amp;21,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=20,"Day "&amp;21,"")</f>
         <v/>
       </c>
       <c r="AT3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=22,"Day "&amp;22,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=21,"Day "&amp;22,"")</f>
         <v/>
       </c>
       <c r="AV3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=23,"Day "&amp;23,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=22,"Day "&amp;23,"")</f>
         <v/>
       </c>
       <c r="AX3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=24,"Day "&amp;24,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=23,"Day "&amp;24,"")</f>
         <v/>
       </c>
       <c r="AZ3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=25,"Day "&amp;25,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=24,"Day "&amp;25,"")</f>
         <v/>
       </c>
       <c r="BB3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=26,"Day "&amp;26,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=25,"Day "&amp;26,"")</f>
         <v/>
       </c>
       <c r="BD3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=27,"Day "&amp;27,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=26,"Day "&amp;27,"")</f>
         <v/>
       </c>
       <c r="BF3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=28,"Day "&amp;28,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=27,"Day "&amp;28,"")</f>
         <v/>
       </c>
       <c r="BH3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=29,"Day "&amp;29,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=28,"Day "&amp;29,"")</f>
         <v/>
       </c>
       <c r="BJ3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=30,"Day "&amp;30,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=29,"Day "&amp;30,"")</f>
         <v/>
       </c>
       <c r="BL3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=31,"Day "&amp;31,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=30,"Day "&amp;31,"")</f>
         <v/>
       </c>
       <c r="BN3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=32,"Day "&amp;32,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=31,"Day "&amp;32,"")</f>
         <v/>
       </c>
       <c r="BP3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=33,"Day "&amp;33,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=32,"Day "&amp;33,"")</f>
         <v/>
       </c>
       <c r="BR3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=34,"Day "&amp;34,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=33,"Day "&amp;34,"")</f>
         <v/>
       </c>
       <c r="BT3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=35,"Day "&amp;35,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=34,"Day "&amp;35,"")</f>
         <v/>
       </c>
       <c r="BV3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=36,"Day "&amp;36,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=35,"Day "&amp;36,"")</f>
         <v/>
       </c>
       <c r="BX3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=37,"Day "&amp;37,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=36,"Day "&amp;37,"")</f>
         <v/>
       </c>
       <c r="BZ3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=38,"Day "&amp;38,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=37,"Day "&amp;38,"")</f>
         <v/>
       </c>
       <c r="CB3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=39,"Day "&amp;39,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=38,"Day "&amp;39,"")</f>
         <v/>
       </c>
       <c r="CD3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=40,"Day "&amp;40,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=39,"Day "&amp;40,"")</f>
         <v/>
       </c>
       <c r="CF3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=41,"Day "&amp;41,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=40,"Day "&amp;41,"")</f>
         <v/>
       </c>
       <c r="CH3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=42,"Day "&amp;42,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=41,"Day "&amp;42,"")</f>
         <v/>
       </c>
       <c r="CJ3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=43,"Day "&amp;43,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=42,"Day "&amp;43,"")</f>
         <v/>
       </c>
       <c r="CL3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=44,"Day "&amp;44,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=43,"Day "&amp;44,"")</f>
         <v/>
       </c>
       <c r="CN3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=45,"Day "&amp;45,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=44,"Day "&amp;45,"")</f>
         <v/>
       </c>
       <c r="CP3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=46,"Day "&amp;46,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=45,"Day "&amp;46,"")</f>
         <v/>
       </c>
       <c r="CR3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=47,"Day "&amp;47,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=46,"Day "&amp;47,"")</f>
         <v/>
       </c>
       <c r="CT3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=48,"Day "&amp;48,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=47,"Day "&amp;48,"")</f>
         <v/>
       </c>
       <c r="CV3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=49,"Day "&amp;49,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=48,"Day "&amp;49,"")</f>
         <v/>
       </c>
       <c r="CX3" s="225">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=50,"Day "&amp;50,"")</f>
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=49,"Day "&amp;50,"")</f>
         <v/>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="128">
       <c r="D4" s="228">
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=0,DASHBOARD!$M$1+0,"")</f>
+        <v/>
+      </c>
+      <c r="F4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=1,DASHBOARD!$M$1+1,"")</f>
         <v/>
       </c>
-      <c r="F4" s="228">
+      <c r="H4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=2,DASHBOARD!$M$1+2,"")</f>
         <v/>
       </c>
-      <c r="H4" s="228">
+      <c r="J4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=3,DASHBOARD!$M$1+3,"")</f>
         <v/>
       </c>
-      <c r="J4" s="228">
+      <c r="L4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=4,DASHBOARD!$M$1+4,"")</f>
         <v/>
       </c>
-      <c r="L4" s="228">
+      <c r="N4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=5,DASHBOARD!$M$1+5,"")</f>
         <v/>
       </c>
-      <c r="N4" s="228">
+      <c r="P4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=6,DASHBOARD!$M$1+6,"")</f>
         <v/>
       </c>
-      <c r="P4" s="228">
+      <c r="R4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=7,DASHBOARD!$M$1+7,"")</f>
         <v/>
       </c>
-      <c r="R4" s="228">
+      <c r="T4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=8,DASHBOARD!$M$1+8,"")</f>
         <v/>
       </c>
-      <c r="T4" s="228">
+      <c r="V4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=9,DASHBOARD!$M$1+9,"")</f>
         <v/>
       </c>
-      <c r="V4" s="228">
+      <c r="X4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=10,DASHBOARD!$M$1+10,"")</f>
         <v/>
       </c>
-      <c r="X4" s="228">
+      <c r="Z4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=11,DASHBOARD!$M$1+11,"")</f>
         <v/>
       </c>
-      <c r="Z4" s="228">
+      <c r="AB4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=12,DASHBOARD!$M$1+12,"")</f>
         <v/>
       </c>
-      <c r="AB4" s="228">
+      <c r="AD4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=13,DASHBOARD!$M$1+13,"")</f>
         <v/>
       </c>
-      <c r="AD4" s="228">
+      <c r="AF4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=14,DASHBOARD!$M$1+14,"")</f>
         <v/>
       </c>
-      <c r="AF4" s="228">
+      <c r="AH4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=15,DASHBOARD!$M$1+15,"")</f>
         <v/>
       </c>
-      <c r="AH4" s="228">
+      <c r="AJ4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=16,DASHBOARD!$M$1+16,"")</f>
         <v/>
       </c>
-      <c r="AJ4" s="228">
+      <c r="AL4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=17,DASHBOARD!$M$1+17,"")</f>
         <v/>
       </c>
-      <c r="AL4" s="228">
+      <c r="AN4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=18,DASHBOARD!$M$1+18,"")</f>
         <v/>
       </c>
-      <c r="AN4" s="228">
+      <c r="AP4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=19,DASHBOARD!$M$1+19,"")</f>
         <v/>
       </c>
-      <c r="AP4" s="228">
+      <c r="AR4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=20,DASHBOARD!$M$1+20,"")</f>
         <v/>
       </c>
-      <c r="AR4" s="228">
+      <c r="AT4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=21,DASHBOARD!$M$1+21,"")</f>
         <v/>
       </c>
-      <c r="AT4" s="228">
+      <c r="AV4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=22,DASHBOARD!$M$1+22,"")</f>
         <v/>
       </c>
-      <c r="AV4" s="228">
+      <c r="AX4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=23,DASHBOARD!$M$1+23,"")</f>
         <v/>
       </c>
-      <c r="AX4" s="228">
+      <c r="AZ4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=24,DASHBOARD!$M$1+24,"")</f>
         <v/>
       </c>
-      <c r="AZ4" s="228">
+      <c r="BB4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=25,DASHBOARD!$M$1+25,"")</f>
         <v/>
       </c>
-      <c r="BB4" s="228">
+      <c r="BD4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=26,DASHBOARD!$M$1+26,"")</f>
         <v/>
       </c>
-      <c r="BD4" s="228">
+      <c r="BF4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=27,DASHBOARD!$M$1+27,"")</f>
         <v/>
       </c>
-      <c r="BF4" s="228">
+      <c r="BH4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=28,DASHBOARD!$M$1+28,"")</f>
         <v/>
       </c>
-      <c r="BH4" s="228">
+      <c r="BJ4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=29,DASHBOARD!$M$1+29,"")</f>
         <v/>
       </c>
-      <c r="BJ4" s="228">
+      <c r="BL4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=30,DASHBOARD!$M$1+30,"")</f>
         <v/>
       </c>
-      <c r="BL4" s="228">
+      <c r="BN4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=31,DASHBOARD!$M$1+31,"")</f>
         <v/>
       </c>
-      <c r="BN4" s="228">
+      <c r="BP4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=32,DASHBOARD!$M$1+32,"")</f>
         <v/>
       </c>
-      <c r="BP4" s="228">
+      <c r="BR4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=33,DASHBOARD!$M$1+33,"")</f>
         <v/>
       </c>
-      <c r="BR4" s="228">
+      <c r="BT4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=34,DASHBOARD!$M$1+34,"")</f>
         <v/>
       </c>
-      <c r="BT4" s="228">
+      <c r="BV4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=35,DASHBOARD!$M$1+35,"")</f>
         <v/>
       </c>
-      <c r="BV4" s="228">
+      <c r="BX4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=36,DASHBOARD!$M$1+36,"")</f>
         <v/>
       </c>
-      <c r="BX4" s="228">
+      <c r="BZ4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=37,DASHBOARD!$M$1+37,"")</f>
         <v/>
       </c>
-      <c r="BZ4" s="228">
+      <c r="CB4" s="228">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=38,DASHBOARD!$M$1+38,"")</f>
         <v/>
       </c>
-      <c r="CB4" s="228">
+      <c r="CD4" s="229">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=39,DASHBOARD!$M$1+39,"")</f>
         <v/>
       </c>
-      <c r="CD4" s="229">
+      <c r="CF4" s="229">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=40,DASHBOARD!$M$1+40,"")</f>
         <v/>
       </c>
-      <c r="CF4" s="229">
+      <c r="CH4" s="229">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=41,DASHBOARD!$M$1+41,"")</f>
         <v/>
       </c>
-      <c r="CH4" s="229">
+      <c r="CJ4" s="229">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=42,DASHBOARD!$M$1+42,"")</f>
         <v/>
       </c>
-      <c r="CJ4" s="229">
+      <c r="CL4" s="229">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=43,DASHBOARD!$M$1+43,"")</f>
         <v/>
       </c>
-      <c r="CL4" s="229">
+      <c r="CN4" s="229">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=44,DASHBOARD!$M$1+44,"")</f>
         <v/>
       </c>
-      <c r="CN4" s="229">
+      <c r="CP4" s="229">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=45,DASHBOARD!$M$1+45,"")</f>
         <v/>
       </c>
-      <c r="CP4" s="229">
+      <c r="CR4" s="229">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=46,DASHBOARD!$M$1+46,"")</f>
         <v/>
       </c>
-      <c r="CR4" s="229">
+      <c r="CT4" s="229">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=47,DASHBOARD!$M$1+47,"")</f>
         <v/>
       </c>
-      <c r="CT4" s="229">
+      <c r="CV4" s="229">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=48,DASHBOARD!$M$1+48,"")</f>
         <v/>
       </c>
-      <c r="CV4" s="229">
+      <c r="CX4" s="229">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=49,DASHBOARD!$M$1+49,"")</f>
-        <v/>
-      </c>
-      <c r="CX4" s="229">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=50,DASHBOARD!$M$1+50,"")</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="10.95" customHeight="1" s="128">
       <c r="D5" s="230">
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=0,"D","")</f>
+        <v/>
+      </c>
+      <c r="E5" s="231">
+        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=0,"T","")</f>
+        <v/>
+      </c>
+      <c r="F5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=1,"D","")</f>
         <v/>
       </c>
-      <c r="E5" s="231">
+      <c r="G5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=1,"T","")</f>
         <v/>
       </c>
-      <c r="F5" s="230">
+      <c r="H5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=2,"D","")</f>
         <v/>
       </c>
-      <c r="G5" s="231">
+      <c r="I5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=2,"T","")</f>
         <v/>
       </c>
-      <c r="H5" s="230">
+      <c r="J5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=3,"D","")</f>
         <v/>
       </c>
-      <c r="I5" s="231">
+      <c r="K5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=3,"T","")</f>
         <v/>
       </c>
-      <c r="J5" s="230">
+      <c r="L5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=4,"D","")</f>
         <v/>
       </c>
-      <c r="K5" s="231">
+      <c r="M5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=4,"T","")</f>
         <v/>
       </c>
-      <c r="L5" s="230">
+      <c r="N5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=5,"D","")</f>
         <v/>
       </c>
-      <c r="M5" s="231">
+      <c r="O5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=5,"T","")</f>
         <v/>
       </c>
-      <c r="N5" s="230">
+      <c r="P5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=6,"D","")</f>
         <v/>
       </c>
-      <c r="O5" s="231">
+      <c r="Q5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=6,"T","")</f>
         <v/>
       </c>
-      <c r="P5" s="230">
+      <c r="R5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=7,"D","")</f>
         <v/>
       </c>
-      <c r="Q5" s="231">
+      <c r="S5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=7,"T","")</f>
         <v/>
       </c>
-      <c r="R5" s="230">
+      <c r="T5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=8,"D","")</f>
         <v/>
       </c>
-      <c r="S5" s="231">
+      <c r="U5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=8,"T","")</f>
         <v/>
       </c>
-      <c r="T5" s="230">
+      <c r="V5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=9,"D","")</f>
         <v/>
       </c>
-      <c r="U5" s="231">
+      <c r="W5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=9,"T","")</f>
         <v/>
       </c>
-      <c r="V5" s="230">
+      <c r="X5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=10,"D","")</f>
         <v/>
       </c>
-      <c r="W5" s="231">
+      <c r="Y5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=10,"T","")</f>
         <v/>
       </c>
-      <c r="X5" s="230">
+      <c r="Z5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=11,"D","")</f>
         <v/>
       </c>
-      <c r="Y5" s="231">
+      <c r="AA5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=11,"T","")</f>
         <v/>
       </c>
-      <c r="Z5" s="230">
+      <c r="AB5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=12,"D","")</f>
         <v/>
       </c>
-      <c r="AA5" s="231">
+      <c r="AC5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=12,"T","")</f>
         <v/>
       </c>
-      <c r="AB5" s="230">
+      <c r="AD5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=13,"D","")</f>
         <v/>
       </c>
-      <c r="AC5" s="231">
+      <c r="AE5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=13,"T","")</f>
         <v/>
       </c>
-      <c r="AD5" s="230">
+      <c r="AF5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=14,"D","")</f>
         <v/>
       </c>
-      <c r="AE5" s="231">
+      <c r="AG5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=14,"T","")</f>
         <v/>
       </c>
-      <c r="AF5" s="230">
+      <c r="AH5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=15,"D","")</f>
         <v/>
       </c>
-      <c r="AG5" s="231">
+      <c r="AI5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=15,"T","")</f>
         <v/>
       </c>
-      <c r="AH5" s="230">
+      <c r="AJ5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=16,"D","")</f>
         <v/>
       </c>
-      <c r="AI5" s="231">
+      <c r="AK5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=16,"T","")</f>
         <v/>
       </c>
-      <c r="AJ5" s="230">
+      <c r="AL5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=17,"D","")</f>
         <v/>
       </c>
-      <c r="AK5" s="231">
+      <c r="AM5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=17,"T","")</f>
         <v/>
       </c>
-      <c r="AL5" s="230">
+      <c r="AN5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=18,"D","")</f>
         <v/>
       </c>
-      <c r="AM5" s="231">
+      <c r="AO5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=18,"T","")</f>
         <v/>
       </c>
-      <c r="AN5" s="230">
+      <c r="AP5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=19,"D","")</f>
         <v/>
       </c>
-      <c r="AO5" s="231">
+      <c r="AQ5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=19,"T","")</f>
         <v/>
       </c>
-      <c r="AP5" s="230">
+      <c r="AR5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=20,"D","")</f>
         <v/>
       </c>
-      <c r="AQ5" s="231">
+      <c r="AS5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=20,"T","")</f>
         <v/>
       </c>
-      <c r="AR5" s="230">
+      <c r="AT5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=21,"D","")</f>
         <v/>
       </c>
-      <c r="AS5" s="231">
+      <c r="AU5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=21,"T","")</f>
         <v/>
       </c>
-      <c r="AT5" s="230">
+      <c r="AV5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=22,"D","")</f>
         <v/>
       </c>
-      <c r="AU5" s="231">
+      <c r="AW5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=22,"T","")</f>
         <v/>
       </c>
-      <c r="AV5" s="230">
+      <c r="AX5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=23,"D","")</f>
         <v/>
       </c>
-      <c r="AW5" s="231">
+      <c r="AY5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=23,"T","")</f>
         <v/>
       </c>
-      <c r="AX5" s="230">
+      <c r="AZ5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=24,"D","")</f>
         <v/>
       </c>
-      <c r="AY5" s="231">
+      <c r="BA5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=24,"T","")</f>
         <v/>
       </c>
-      <c r="AZ5" s="230">
+      <c r="BB5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=25,"D","")</f>
         <v/>
       </c>
-      <c r="BA5" s="231">
+      <c r="BC5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=25,"T","")</f>
         <v/>
       </c>
-      <c r="BB5" s="230">
+      <c r="BD5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=26,"D","")</f>
         <v/>
       </c>
-      <c r="BC5" s="231">
+      <c r="BE5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=26,"T","")</f>
         <v/>
       </c>
-      <c r="BD5" s="230">
+      <c r="BF5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=27,"D","")</f>
         <v/>
       </c>
-      <c r="BE5" s="231">
+      <c r="BG5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=27,"T","")</f>
         <v/>
       </c>
-      <c r="BF5" s="230">
+      <c r="BH5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=28,"D","")</f>
         <v/>
       </c>
-      <c r="BG5" s="231">
+      <c r="BI5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=28,"T","")</f>
         <v/>
       </c>
-      <c r="BH5" s="230">
+      <c r="BJ5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=29,"D","")</f>
         <v/>
       </c>
-      <c r="BI5" s="231">
+      <c r="BK5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=29,"T","")</f>
         <v/>
       </c>
-      <c r="BJ5" s="230">
+      <c r="BL5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=30,"D","")</f>
         <v/>
       </c>
-      <c r="BK5" s="231">
+      <c r="BM5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=30,"T","")</f>
         <v/>
       </c>
-      <c r="BL5" s="230">
+      <c r="BN5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=31,"D","")</f>
         <v/>
       </c>
-      <c r="BM5" s="231">
+      <c r="BO5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=31,"T","")</f>
         <v/>
       </c>
-      <c r="BN5" s="230">
+      <c r="BP5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=32,"D","")</f>
         <v/>
       </c>
-      <c r="BO5" s="231">
+      <c r="BQ5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=32,"T","")</f>
         <v/>
       </c>
-      <c r="BP5" s="230">
+      <c r="BR5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=33,"D","")</f>
         <v/>
       </c>
-      <c r="BQ5" s="231">
+      <c r="BS5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=33,"T","")</f>
         <v/>
       </c>
-      <c r="BR5" s="230">
+      <c r="BT5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=34,"D","")</f>
         <v/>
       </c>
-      <c r="BS5" s="231">
+      <c r="BU5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=34,"T","")</f>
         <v/>
       </c>
-      <c r="BT5" s="230">
+      <c r="BV5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=35,"D","")</f>
         <v/>
       </c>
-      <c r="BU5" s="231">
+      <c r="BW5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=35,"T","")</f>
         <v/>
       </c>
-      <c r="BV5" s="230">
+      <c r="BX5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=36,"D","")</f>
         <v/>
       </c>
-      <c r="BW5" s="231">
+      <c r="BY5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=36,"T","")</f>
         <v/>
       </c>
-      <c r="BX5" s="230">
+      <c r="BZ5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=37,"D","")</f>
         <v/>
       </c>
-      <c r="BY5" s="231">
+      <c r="CA5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=37,"T","")</f>
         <v/>
       </c>
-      <c r="BZ5" s="230">
+      <c r="CB5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=38,"D","")</f>
         <v/>
       </c>
-      <c r="CA5" s="231">
+      <c r="CC5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=38,"T","")</f>
         <v/>
       </c>
-      <c r="CB5" s="230">
+      <c r="CD5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=39,"D","")</f>
         <v/>
       </c>
-      <c r="CC5" s="231">
+      <c r="CE5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=39,"T","")</f>
         <v/>
       </c>
-      <c r="CD5" s="230">
+      <c r="CF5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=40,"D","")</f>
         <v/>
       </c>
-      <c r="CE5" s="231">
+      <c r="CG5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=40,"T","")</f>
         <v/>
       </c>
-      <c r="CF5" s="230">
+      <c r="CH5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=41,"D","")</f>
         <v/>
       </c>
-      <c r="CG5" s="231">
+      <c r="CI5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=41,"T","")</f>
         <v/>
       </c>
-      <c r="CH5" s="230">
+      <c r="CJ5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=42,"D","")</f>
         <v/>
       </c>
-      <c r="CI5" s="231">
+      <c r="CK5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=42,"T","")</f>
         <v/>
       </c>
-      <c r="CJ5" s="230">
+      <c r="CL5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=43,"D","")</f>
         <v/>
       </c>
-      <c r="CK5" s="231">
+      <c r="CM5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=43,"T","")</f>
         <v/>
       </c>
-      <c r="CL5" s="230">
+      <c r="CN5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=44,"D","")</f>
         <v/>
       </c>
-      <c r="CM5" s="231">
+      <c r="CO5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=44,"T","")</f>
         <v/>
       </c>
-      <c r="CN5" s="230">
+      <c r="CP5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=45,"D","")</f>
         <v/>
       </c>
-      <c r="CO5" s="231">
+      <c r="CQ5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=45,"T","")</f>
         <v/>
       </c>
-      <c r="CP5" s="230">
+      <c r="CR5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=46,"D","")</f>
         <v/>
       </c>
-      <c r="CQ5" s="231">
+      <c r="CS5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=46,"T","")</f>
         <v/>
       </c>
-      <c r="CR5" s="230">
+      <c r="CT5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=47,"D","")</f>
         <v/>
       </c>
-      <c r="CS5" s="231">
+      <c r="CU5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=47,"T","")</f>
         <v/>
       </c>
-      <c r="CT5" s="230">
+      <c r="CV5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=48,"D","")</f>
         <v/>
       </c>
-      <c r="CU5" s="231">
+      <c r="CW5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=48,"T","")</f>
         <v/>
       </c>
-      <c r="CV5" s="230">
+      <c r="CX5" s="230">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=49,"D","")</f>
         <v/>
       </c>
-      <c r="CW5" s="231">
+      <c r="CY5" s="231">
         <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=49,"T","")</f>
-        <v/>
-      </c>
-      <c r="CX5" s="230">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=50,"D","")</f>
-        <v/>
-      </c>
-      <c r="CY5" s="231">
-        <f>IF(DASHBOARD!$M$2-DASHBOARD!$M$1&gt;=50,"T","")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Layover CF rebuilt clean — Day38=24Aug, bars fixed
</commit_message>
<xml_diff>
--- a/uploads/HZ-ASD_C2_6Y_CABIN_WP_TRACKER.xlsx
+++ b/uploads/HZ-ASD_C2_6Y_CABIN_WP_TRACKER.xlsx
@@ -41815,40 +41815,40 @@
   </mergeCells>
   <conditionalFormatting sqref="D19:CY19">
     <cfRule type="expression" priority="11" dxfId="103" stopIfTrue="1">
-      <formula>DASHBOARD!$M$1+1+INT((COLUMN()-4)/2)=INT($B$19)</formula>
+      <formula>(DASHBOARD!$M$1+INT((COLUMN()-4)/2))=INT($B$19)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D25:CY25">
     <cfRule type="expression" priority="12" dxfId="103" stopIfTrue="1">
-      <formula>DASHBOARD!$M$1+1+INT((COLUMN()-4)/2)=INT($B$25)</formula>
+      <formula>(DASHBOARD!$M$1+INT((COLUMN()-4)/2))=INT($B$25)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D6:CY38">
     <cfRule type="expression" priority="13" dxfId="104" stopIfTrue="1">
-      <formula>AND(ISNUMBER($B6),(DASHBOARD!$M$1+1+(COLUMN()-4)/2)&gt;=(INT($B6)+IF(MOD($B6,1)&lt;0.5,0,0.5)),(DASHBOARD!$M$1+1+(COLUMN()-4)/2)&lt;(INT(IF(ISNUMBER($C6),$C6,$B6))+IF(MOD(IF(ISNUMBER($C6),$C6,$B6),1)=0,1,IF(MOD(IF(ISNUMBER($C6),$C6,$B6),1)&lt;=0.5,0.5,1))))</formula>
+      <formula>AND(ISNUMBER($B6),(DASHBOARD!$M$1+(COLUMN()-4)/2)&gt;=(INT($B6)+IF(MOD($B6,1)&lt;0.5,0,0.5)),(DASHBOARD!$M$1+(COLUMN()-4)/2)&lt;(INT(IF(ISNUMBER($C6),$C6,$B6))+IF(MOD(IF(ISNUMBER($C6),$C6,$B6),1)=0,1,IF(MOD(IF(ISNUMBER($C6),$C6,$B6),1)&lt;=0.5,0.5,1))))</formula>
     </cfRule>
     <cfRule type="expression" priority="14" dxfId="105">
-      <formula>AND(MOD(COLUMN(),2)=0,DASHBOARD!$M$1+1+INT((COLUMN()-4)/2)=INT($B$19))</formula>
+      <formula>AND(MOD(COLUMN(),2)=0,(DASHBOARD!$M$1+INT((COLUMN()-4)/2))=INT($B$19))</formula>
     </cfRule>
     <cfRule type="expression" priority="15" dxfId="106">
-      <formula>AND(MOD(COLUMN(),2)=1,DASHBOARD!$M$1+1+INT((COLUMN()-4)/2)=INT($B$25))</formula>
+      <formula>AND(MOD(COLUMN(),2)=1,(DASHBOARD!$M$1+INT((COLUMN()-4)/2))=INT($B$25))</formula>
     </cfRule>
     <cfRule type="expression" priority="16" dxfId="110" stopIfTrue="1">
-      <formula>DASHBOARD!$M$1+1+INT((COLUMN()-4)/2)&gt;DASHBOARD!$M$2</formula>
+      <formula>(DASHBOARD!$M$1+INT((COLUMN()-4)/2))&gt;DASHBOARD!$M$2</formula>
+    </cfRule>
+    <cfRule type="expression" priority="17" dxfId="107">
+      <formula>(DASHBOARD!$M$1+INT((COLUMN()-4)/2))=TODAY()</formula>
     </cfRule>
     <cfRule type="expression" priority="18" dxfId="108">
-      <formula>DASHBOARD!$M$1+1+INT((COLUMN()-4)/2)=DASHBOARD!$M$2</formula>
+      <formula>(DASHBOARD!$M$1+INT((COLUMN()-4)/2))=DASHBOARD!$M$2</formula>
     </cfRule>
     <cfRule type="expression" priority="19" dxfId="109">
-      <formula>OR(WEEKDAY(DASHBOARD!$M$1+1+INT((COLUMN()-4)/2),2)=5,WEEKDAY(DASHBOARD!$M$1+1+INT((COLUMN()-4)/2),2)=6)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="11" dxfId="107">
-      <formula>DASHBOARD!$M$1+INT((COLUMN()-4)/2)=TODAY()</formula>
+      <formula>OR(WEEKDAY((DASHBOARD!$M$1+INT((COLUMN()-4)/2)),2)=5,WEEKDAY((DASHBOARD!$M$1+INT((COLUMN()-4)/2)),2)=6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D3:CY5">
     <cfRule type="expression" priority="20" dxfId="111" stopIfTrue="1">
-      <formula>DASHBOARD!$M$1+1+INT((COLUMN()-4)/2)&gt;DASHBOARD!$M$2</formula>
+      <formula>(DASHBOARD!$M$1+INT((COLUMN()-4)/2))&gt;DASHBOARD!$M$2</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Compatibility: MINIFS → AGGREGATE (Excel 2010+)
</commit_message>
<xml_diff>
--- a/uploads/HZ-ASD_C2_6Y_CABIN_WP_TRACKER.xlsx
+++ b/uploads/HZ-ASD_C2_6Y_CABIN_WP_TRACKER.xlsx
@@ -35158,7 +35158,7 @@
     </row>
     <row r="11" ht="18" customHeight="1" s="128">
       <c r="A11" s="292">
-        <f>IFERROR("📅 Next: "&amp;INDEX(LAYOVER!$A$41:$A$48,MATCH(_xludf.MINIFS(LAYOVER!$B$41:$B$48,LAYOVER!$B$41:$B$48,"&gt;="&amp;TODAY()),LAYOVER!$B$41:$B$48,0))&amp;IF(_xludf.MINIFS(LAYOVER!$B$41:$B$48,LAYOVER!$B$41:$B$48,"&gt;="&amp;TODAY())=TODAY()," — TODAY"," in "&amp;(_xludf.MINIFS(LAYOVER!$B$41:$B$48,LAYOVER!$B$41:$B$48,"&gt;="&amp;TODAY())-TODAY())&amp;" day(s)"),"📅 no upcoming milestone set")</f>
+        <f>IFERROR("📅 Next: "&amp;INDEX('LAYOVER'!$A$41:$A$48,MATCH(AGGREGATE(15,6,'LAYOVER'!$B$41:$B$48/('LAYOVER'!$B$41:$B$48&gt;=TODAY()),1),'LAYOVER'!$B$41:$B$48,0))&amp;IF(AGGREGATE(15,6,'LAYOVER'!$B$41:$B$48/('LAYOVER'!$B$41:$B$48&gt;=TODAY()),1)=TODAY()," — TODAY"," in "&amp;(AGGREGATE(15,6,'LAYOVER'!$B$41:$B$48/('LAYOVER'!$B$41:$B$48&gt;=TODAY()),1)-TODAY())&amp;" day(s)"),"📅 no upcoming milestone set")</f>
         <v/>
       </c>
     </row>
@@ -36407,6 +36407,7 @@
         <v/>
       </c>
     </row>
+    <row r="65"/>
     <row r="66" ht="18" customHeight="1" s="128">
       <c r="A66" s="239" t="inlineStr">
         <is>
@@ -41584,6 +41585,7 @@
       <c r="CX38" s="232" t="n"/>
       <c r="CY38" s="234" t="n"/>
     </row>
+    <row r="39"/>
     <row r="40" ht="16" customHeight="1" s="128">
       <c r="A40" s="239" t="inlineStr">
         <is>
@@ -59810,7 +59812,7 @@
         </is>
       </c>
       <c r="H9" s="183">
-        <f>IFERROR("📅 Next: "&amp;INDEX(LAYOVER!$A$41:$A$48,MATCH(_xludf.MINIFS(LAYOVER!$B$41:$B$48,LAYOVER!$B$41:$B$48,"&gt;="&amp;TODAY()),LAYOVER!$B$41:$B$48,0))&amp;IF(_xludf.MINIFS(LAYOVER!$B$41:$B$48,LAYOVER!$B$41:$B$48,"&gt;="&amp;TODAY())=TODAY()," — TODAY"," in "&amp;(_xludf.MINIFS(LAYOVER!$B$41:$B$48,LAYOVER!$B$41:$B$48,"&gt;="&amp;TODAY())-TODAY())&amp;" day(s)"),"📅 no upcoming milestone set")</f>
+        <f>IFERROR("📅 Next: "&amp;INDEX('LAYOVER'!$A$41:$A$48,MATCH(AGGREGATE(15,6,'LAYOVER'!$B$41:$B$48/('LAYOVER'!$B$41:$B$48&gt;=TODAY()),1),'LAYOVER'!$B$41:$B$48,0))&amp;IF(AGGREGATE(15,6,'LAYOVER'!$B$41:$B$48/('LAYOVER'!$B$41:$B$48&gt;=TODAY()),1)=TODAY()," — TODAY"," in "&amp;(AGGREGATE(15,6,'LAYOVER'!$B$41:$B$48/('LAYOVER'!$B$41:$B$48&gt;=TODAY()),1)-TODAY())&amp;" day(s)"),"📅 no upcoming milestone set")</f>
         <v/>
       </c>
       <c r="L9" s="101" t="n"/>
@@ -59907,6 +59909,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="18" customHeight="1" s="128">
       <c r="A18" s="185" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix 809 MH cells: date-format contamination → clean hour numbers
</commit_message>
<xml_diff>
--- a/uploads/HZ-ASD_C2_6Y_CABIN_WP_TRACKER.xlsx
+++ b/uploads/HZ-ASD_C2_6Y_CABIN_WP_TRACKER.xlsx
@@ -17521,7 +17521,7 @@
       </c>
       <c r="L196" s="100" t="n"/>
       <c r="M196" s="276" t="n"/>
-      <c r="N196" s="327" t="n">
+      <c r="N196" s="326" t="n">
         <v>12</v>
       </c>
       <c r="O196" s="327" t="n"/>
@@ -17570,7 +17570,7 @@
       </c>
       <c r="L197" s="100" t="n"/>
       <c r="M197" s="276" t="n"/>
-      <c r="N197" s="327" t="n">
+      <c r="N197" s="326" t="n">
         <v>120</v>
       </c>
       <c r="O197" s="327" t="n"/>
@@ -17623,7 +17623,7 @@
       </c>
       <c r="L198" s="100" t="n"/>
       <c r="M198" s="276" t="n"/>
-      <c r="N198" s="327" t="n">
+      <c r="N198" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O198" s="327" t="n"/>
@@ -17672,7 +17672,7 @@
       </c>
       <c r="L199" s="100" t="n"/>
       <c r="M199" s="276" t="n"/>
-      <c r="N199" s="327" t="n">
+      <c r="N199" s="326" t="n">
         <v>22</v>
       </c>
       <c r="O199" s="327" t="n"/>
@@ -17721,7 +17721,7 @@
       </c>
       <c r="L200" s="100" t="n"/>
       <c r="M200" s="276" t="n"/>
-      <c r="N200" s="327" t="n">
+      <c r="N200" s="326" t="n">
         <v>5</v>
       </c>
       <c r="O200" s="327" t="n"/>
@@ -17770,7 +17770,7 @@
       </c>
       <c r="L201" s="100" t="n"/>
       <c r="M201" s="276" t="n"/>
-      <c r="N201" s="327" t="n">
+      <c r="N201" s="326" t="n">
         <v>3</v>
       </c>
       <c r="O201" s="327" t="n"/>
@@ -17819,7 +17819,7 @@
       </c>
       <c r="L202" s="100" t="n"/>
       <c r="M202" s="276" t="n"/>
-      <c r="N202" s="327" t="n">
+      <c r="N202" s="326" t="n">
         <v>3</v>
       </c>
       <c r="O202" s="327" t="n"/>
@@ -17868,7 +17868,7 @@
       </c>
       <c r="L203" s="100" t="n"/>
       <c r="M203" s="276" t="n"/>
-      <c r="N203" s="327" t="n">
+      <c r="N203" s="326" t="n">
         <v>12</v>
       </c>
       <c r="O203" s="327" t="n"/>
@@ -17917,7 +17917,7 @@
       </c>
       <c r="L204" s="100" t="n"/>
       <c r="M204" s="276" t="n"/>
-      <c r="N204" s="327" t="n">
+      <c r="N204" s="326" t="n">
         <v>3</v>
       </c>
       <c r="O204" s="327" t="n"/>
@@ -17966,7 +17966,7 @@
       </c>
       <c r="L205" s="100" t="n"/>
       <c r="M205" s="276" t="n"/>
-      <c r="N205" s="327" t="n">
+      <c r="N205" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O205" s="327" t="n"/>
@@ -18156,7 +18156,7 @@
       </c>
       <c r="L209" s="100" t="n"/>
       <c r="M209" s="276" t="n"/>
-      <c r="N209" s="327" t="n">
+      <c r="N209" s="326" t="n">
         <v>24</v>
       </c>
       <c r="O209" s="327" t="n"/>
@@ -18209,7 +18209,7 @@
       </c>
       <c r="L210" s="100" t="n"/>
       <c r="M210" s="276" t="n"/>
-      <c r="N210" s="327" t="n">
+      <c r="N210" s="326" t="n">
         <v>24</v>
       </c>
       <c r="O210" s="327" t="n"/>
@@ -18262,7 +18262,7 @@
       </c>
       <c r="L211" s="100" t="n"/>
       <c r="M211" s="276" t="n"/>
-      <c r="N211" s="327" t="n">
+      <c r="N211" s="326" t="n">
         <v>12</v>
       </c>
       <c r="O211" s="327" t="n"/>
@@ -18311,7 +18311,7 @@
       </c>
       <c r="L212" s="100" t="n"/>
       <c r="M212" s="276" t="n"/>
-      <c r="N212" s="327" t="n">
+      <c r="N212" s="326" t="n">
         <v>6</v>
       </c>
       <c r="O212" s="327" t="n"/>
@@ -18407,7 +18407,7 @@
       <c r="K214" s="9" t="n"/>
       <c r="L214" s="100" t="n"/>
       <c r="M214" s="276" t="n"/>
-      <c r="N214" s="327" t="n">
+      <c r="N214" s="326" t="n">
         <v>1.5</v>
       </c>
       <c r="O214" s="327" t="n"/>
@@ -18456,7 +18456,7 @@
       <c r="M215" s="276" t="n">
         <v>46222</v>
       </c>
-      <c r="N215" s="327" t="n">
+      <c r="N215" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O215" s="327" t="n"/>
@@ -18505,7 +18505,7 @@
       <c r="K216" s="9" t="n"/>
       <c r="L216" s="100" t="n"/>
       <c r="M216" s="276" t="n"/>
-      <c r="N216" s="327" t="n">
+      <c r="N216" s="326" t="n">
         <v>24</v>
       </c>
       <c r="O216" s="327" t="n"/>
@@ -18550,7 +18550,7 @@
       <c r="K217" s="9" t="n"/>
       <c r="L217" s="100" t="n"/>
       <c r="M217" s="276" t="n"/>
-      <c r="N217" s="327" t="n">
+      <c r="N217" s="326" t="n">
         <v>1</v>
       </c>
       <c r="O217" s="327" t="n"/>
@@ -18595,7 +18595,7 @@
       <c r="K218" s="9" t="n"/>
       <c r="L218" s="100" t="n"/>
       <c r="M218" s="276" t="n"/>
-      <c r="N218" s="327" t="n">
+      <c r="N218" s="326" t="n">
         <v>6</v>
       </c>
       <c r="O218" s="327" t="n"/>
@@ -18640,7 +18640,7 @@
       <c r="K219" s="9" t="n"/>
       <c r="L219" s="100" t="n"/>
       <c r="M219" s="276" t="n"/>
-      <c r="N219" s="327" t="n">
+      <c r="N219" s="326" t="n">
         <v>3.5</v>
       </c>
       <c r="O219" s="327" t="n"/>
@@ -18685,7 +18685,7 @@
       <c r="K220" s="9" t="n"/>
       <c r="L220" s="100" t="n"/>
       <c r="M220" s="276" t="n"/>
-      <c r="N220" s="327" t="n">
+      <c r="N220" s="326" t="n">
         <v>16</v>
       </c>
       <c r="O220" s="327" t="n"/>
@@ -18736,7 +18736,7 @@
       <c r="K221" s="9" t="n"/>
       <c r="L221" s="100" t="n"/>
       <c r="M221" s="276" t="n"/>
-      <c r="N221" s="327" t="n">
+      <c r="N221" s="326" t="n">
         <v>1.5</v>
       </c>
       <c r="O221" s="327" t="n"/>
@@ -18867,7 +18867,7 @@
       <c r="K224" s="9" t="n"/>
       <c r="L224" s="100" t="n"/>
       <c r="M224" s="276" t="n"/>
-      <c r="N224" s="327" t="n">
+      <c r="N224" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O224" s="327" t="n"/>
@@ -18914,7 +18914,7 @@
       <c r="K225" s="9" t="n"/>
       <c r="L225" s="100" t="n"/>
       <c r="M225" s="276" t="n"/>
-      <c r="N225" s="327" t="n">
+      <c r="N225" s="326" t="n">
         <v>2.8</v>
       </c>
       <c r="O225" s="327" t="n"/>
@@ -18961,7 +18961,7 @@
       <c r="K226" s="9" t="n"/>
       <c r="L226" s="100" t="n"/>
       <c r="M226" s="276" t="n"/>
-      <c r="N226" s="327" t="n">
+      <c r="N226" s="326" t="n">
         <v>5.9</v>
       </c>
       <c r="O226" s="327" t="n"/>
@@ -19049,7 +19049,7 @@
       <c r="K228" s="9" t="n"/>
       <c r="L228" s="100" t="n"/>
       <c r="M228" s="276" t="n"/>
-      <c r="N228" s="327" t="n">
+      <c r="N228" s="326" t="n">
         <v>3</v>
       </c>
       <c r="O228" s="327" t="n"/>
@@ -19094,7 +19094,7 @@
       <c r="K229" s="9" t="n"/>
       <c r="L229" s="100" t="n"/>
       <c r="M229" s="276" t="n"/>
-      <c r="N229" s="327" t="n">
+      <c r="N229" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O229" s="327" t="n"/>
@@ -19139,7 +19139,7 @@
       <c r="K230" s="9" t="n"/>
       <c r="L230" s="100" t="n"/>
       <c r="M230" s="276" t="n"/>
-      <c r="N230" s="327" t="n">
+      <c r="N230" s="326" t="n">
         <v>6</v>
       </c>
       <c r="O230" s="327" t="n"/>
@@ -19184,7 +19184,7 @@
       <c r="K231" s="9" t="n"/>
       <c r="L231" s="100" t="n"/>
       <c r="M231" s="276" t="n"/>
-      <c r="N231" s="327" t="n">
+      <c r="N231" s="326" t="n">
         <v>6</v>
       </c>
       <c r="O231" s="327" t="n"/>
@@ -19229,7 +19229,7 @@
       <c r="K232" s="9" t="n"/>
       <c r="L232" s="100" t="n"/>
       <c r="M232" s="276" t="n"/>
-      <c r="N232" s="327" t="n">
+      <c r="N232" s="326" t="n">
         <v>5</v>
       </c>
       <c r="O232" s="327" t="n"/>
@@ -19274,7 +19274,7 @@
       <c r="K233" s="9" t="n"/>
       <c r="L233" s="100" t="n"/>
       <c r="M233" s="276" t="n"/>
-      <c r="N233" s="327" t="n">
+      <c r="N233" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O233" s="327" t="n"/>
@@ -19319,7 +19319,7 @@
       <c r="K234" s="9" t="n"/>
       <c r="L234" s="100" t="n"/>
       <c r="M234" s="276" t="n"/>
-      <c r="N234" s="327" t="n">
+      <c r="N234" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O234" s="327" t="n"/>
@@ -19364,7 +19364,7 @@
       <c r="K235" s="9" t="n"/>
       <c r="L235" s="100" t="n"/>
       <c r="M235" s="276" t="n"/>
-      <c r="N235" s="327" t="n">
+      <c r="N235" s="326" t="n">
         <v>15</v>
       </c>
       <c r="O235" s="327" t="n"/>
@@ -19460,7 +19460,7 @@
       <c r="K237" s="9" t="n"/>
       <c r="L237" s="100" t="n"/>
       <c r="M237" s="276" t="n"/>
-      <c r="N237" s="327" t="n">
+      <c r="N237" s="326" t="n">
         <v>8</v>
       </c>
       <c r="O237" s="327" t="n"/>
@@ -19877,7 +19877,7 @@
       <c r="K246" s="9" t="n"/>
       <c r="L246" s="100" t="n"/>
       <c r="M246" s="276" t="n"/>
-      <c r="N246" s="327" t="n">
+      <c r="N246" s="326" t="n">
         <v>8.5</v>
       </c>
       <c r="O246" s="327" t="n"/>
@@ -19922,7 +19922,7 @@
       <c r="K247" s="9" t="n"/>
       <c r="L247" s="100" t="n"/>
       <c r="M247" s="276" t="n"/>
-      <c r="N247" s="327" t="n">
+      <c r="N247" s="326" t="n">
         <v>6</v>
       </c>
       <c r="O247" s="327" t="n"/>
@@ -19967,7 +19967,7 @@
       <c r="K248" s="9" t="n"/>
       <c r="L248" s="100" t="n"/>
       <c r="M248" s="276" t="n"/>
-      <c r="N248" s="327" t="n">
+      <c r="N248" s="326" t="n">
         <v>12</v>
       </c>
       <c r="O248" s="327" t="n"/>
@@ -20012,7 +20012,7 @@
       <c r="K249" s="9" t="n"/>
       <c r="L249" s="100" t="n"/>
       <c r="M249" s="276" t="n"/>
-      <c r="N249" s="327" t="n">
+      <c r="N249" s="326" t="n">
         <v>3</v>
       </c>
       <c r="O249" s="327" t="n"/>
@@ -20057,7 +20057,7 @@
       <c r="K250" s="9" t="n"/>
       <c r="L250" s="100" t="n"/>
       <c r="M250" s="276" t="n"/>
-      <c r="N250" s="327" t="n">
+      <c r="N250" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O250" s="327" t="n"/>
@@ -20102,7 +20102,7 @@
       <c r="K251" s="9" t="n"/>
       <c r="L251" s="100" t="n"/>
       <c r="M251" s="276" t="n"/>
-      <c r="N251" s="327" t="n">
+      <c r="N251" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O251" s="327" t="n"/>
@@ -20147,7 +20147,7 @@
       <c r="K252" s="9" t="n"/>
       <c r="L252" s="100" t="n"/>
       <c r="M252" s="276" t="n"/>
-      <c r="N252" s="327" t="n">
+      <c r="N252" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O252" s="327" t="n"/>
@@ -20235,7 +20235,7 @@
       <c r="K254" s="9" t="n"/>
       <c r="L254" s="100" t="n"/>
       <c r="M254" s="276" t="n"/>
-      <c r="N254" s="327" t="n">
+      <c r="N254" s="326" t="n">
         <v>4</v>
       </c>
       <c r="O254" s="327" t="n"/>
@@ -20323,7 +20323,7 @@
       <c r="K256" s="9" t="n"/>
       <c r="L256" s="100" t="n"/>
       <c r="M256" s="276" t="n"/>
-      <c r="N256" s="327" t="n">
+      <c r="N256" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O256" s="327" t="n"/>
@@ -20411,7 +20411,7 @@
       <c r="K258" s="9" t="n"/>
       <c r="L258" s="100" t="n"/>
       <c r="M258" s="276" t="n"/>
-      <c r="N258" s="327" t="n">
+      <c r="N258" s="326" t="n">
         <v>4</v>
       </c>
       <c r="O258" s="327" t="n"/>
@@ -20456,7 +20456,7 @@
       <c r="K259" s="9" t="n"/>
       <c r="L259" s="100" t="n"/>
       <c r="M259" s="276" t="n"/>
-      <c r="N259" s="327" t="n">
+      <c r="N259" s="326" t="n">
         <v>6</v>
       </c>
       <c r="O259" s="327" t="n"/>
@@ -20501,7 +20501,7 @@
       <c r="K260" s="9" t="n"/>
       <c r="L260" s="100" t="n"/>
       <c r="M260" s="276" t="n"/>
-      <c r="N260" s="327" t="n">
+      <c r="N260" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O260" s="327" t="n"/>
@@ -20546,7 +20546,7 @@
       <c r="K261" s="9" t="n"/>
       <c r="L261" s="100" t="n"/>
       <c r="M261" s="276" t="n"/>
-      <c r="N261" s="327" t="n">
+      <c r="N261" s="326" t="n">
         <v>3</v>
       </c>
       <c r="O261" s="327" t="n"/>
@@ -20591,7 +20591,7 @@
       <c r="K262" s="9" t="n"/>
       <c r="L262" s="100" t="n"/>
       <c r="M262" s="276" t="n"/>
-      <c r="N262" s="327" t="n">
+      <c r="N262" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O262" s="327" t="n"/>
@@ -20636,7 +20636,7 @@
       <c r="K263" s="9" t="n"/>
       <c r="L263" s="100" t="n"/>
       <c r="M263" s="276" t="n"/>
-      <c r="N263" s="327" t="n">
+      <c r="N263" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O263" s="327" t="n"/>
@@ -20681,7 +20681,7 @@
       <c r="K264" s="9" t="n"/>
       <c r="L264" s="100" t="n"/>
       <c r="M264" s="276" t="n"/>
-      <c r="N264" s="327" t="n">
+      <c r="N264" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O264" s="327" t="n"/>
@@ -20726,7 +20726,7 @@
       <c r="K265" s="9" t="n"/>
       <c r="L265" s="100" t="n"/>
       <c r="M265" s="276" t="n"/>
-      <c r="N265" s="327" t="n">
+      <c r="N265" s="326" t="n">
         <v>2</v>
       </c>
       <c r="O265" s="327" t="n"/>

</xml_diff>